<commit_message>
Business card: the extension in a field of its own beside the phone, the phone taking only what a number is written with and checked
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/UMO_business-cards_template.xlsx
+++ b/public/downloads/UMO_business-cards_template.xlsx
@@ -55,7 +55,8 @@
     <col min="2" max="2" width="26" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="34" customWidth="1" style="3"/>
-    <col min="5" max="5" width="30" customWidth="1" style="3"/>
+    <col min="5" max="5" width="24" customWidth="1" style="3"/>
+    <col min="6" max="6" width="14" customWidth="1" style="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -84,6 +85,11 @@
           <t xml:space="preserve">Телефон</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr" s="1">
+        <is>
+          <t xml:space="preserve">Добавочный</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr" s="2">
@@ -108,7 +114,12 @@
       </c>
       <c r="E2" t="inlineStr" s="4">
         <is>
-          <t xml:space="preserve">+7 495 000 00 00 доб. 123</t>
+          <t xml:space="preserve">+7 495 000 00 00</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr" s="4">
+        <is>
+          <t xml:space="preserve">123</t>
         </is>
       </c>
     </row>

</xml_diff>